<commit_message>
Added min and max to summary stats
</commit_message>
<xml_diff>
--- a/SummaryStats.xlsx
+++ b/SummaryStats.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Research\00. FishLab\04. Project Folders\Cassandra\LargeSturgeonData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\home.tacoma.uw.edu\cdonatel$\GitHub\Korneisel_TetNecks_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7886B907-AB94-4D03-AB53-B69BC7174112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A41484-4CA5-4F7D-B43F-A1B07B931422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{91481A77-D1F8-4675-95E4-40E8596B26D3}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{91481A77-D1F8-4675-95E4-40E8596B26D3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Roune01" sheetId="1" r:id="rId1"/>
+    <sheet name="Round02" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="29">
   <si>
     <t>column</t>
   </si>
@@ -118,12 +119,18 @@
   <si>
     <t>Torsional Stiffness (GJL, Nm)</t>
   </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,8 +168,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -172,6 +203,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -188,24 +225,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -213,22 +250,76 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -579,7 +670,7 @@
     <col min="14" max="14" width="11" style="6" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="4" style="6" customWidth="1"/>
     <col min="16" max="16" width="4.42578125" style="7" customWidth="1"/>
-    <col min="17" max="17" width="7.42578125" style="15" customWidth="1"/>
+    <col min="17" max="17" width="7.42578125" style="6" customWidth="1"/>
     <col min="18" max="18" width="15" style="6" customWidth="1"/>
     <col min="19" max="19" width="7.140625" style="6" customWidth="1"/>
     <col min="20" max="21" width="11" style="6" bestFit="1" customWidth="1"/>
@@ -1216,7 +1307,7 @@
       <c r="J13" s="4"/>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
-      <c r="Q13" s="15" t="s">
+      <c r="Q13" s="6" t="s">
         <v>25</v>
       </c>
       <c r="R13" s="3"/>
@@ -1687,7 +1778,7 @@
         <v>7</v>
       </c>
       <c r="P23" s="9"/>
-      <c r="Q23" s="15" t="s">
+      <c r="Q23" s="6" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2100,7 +2191,7 @@
         <v>9</v>
       </c>
       <c r="P33" s="9"/>
-      <c r="Q33" s="15" t="s">
+      <c r="Q33" s="6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3023,4 +3114,2843 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F1865B8-B9DB-45A0-9665-E04D44EB77EE}">
+  <dimension ref="A1:AC49"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5" style="15" customWidth="1"/>
+    <col min="2" max="3" width="9.140625" style="15"/>
+    <col min="4" max="6" width="11.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.85546875" style="15" customWidth="1"/>
+    <col min="8" max="9" width="11.140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4" style="30" customWidth="1"/>
+    <col min="11" max="11" width="5.5703125" style="15" customWidth="1"/>
+    <col min="12" max="13" width="9.140625" style="15"/>
+    <col min="14" max="16" width="11" style="15" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="4.7109375" style="15" customWidth="1"/>
+    <col min="18" max="18" width="10.5703125" style="15" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.140625" style="15" customWidth="1"/>
+    <col min="20" max="20" width="4.42578125" style="30" customWidth="1"/>
+    <col min="21" max="21" width="5.5703125" style="15" customWidth="1"/>
+    <col min="22" max="22" width="9.140625" style="15"/>
+    <col min="23" max="23" width="7.7109375" style="15" customWidth="1"/>
+    <col min="24" max="25" width="11" style="15" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="6.85546875" style="15" customWidth="1"/>
+    <col min="28" max="29" width="9.28515625" style="15" bestFit="1" customWidth="1"/>
+    <col min="30" max="16384" width="9.140625" style="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="32"/>
+      <c r="T1" s="33"/>
+      <c r="U1" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="V1" s="35"/>
+      <c r="W1" s="35"/>
+      <c r="X1" s="35"/>
+      <c r="Y1" s="35"/>
+      <c r="Z1" s="35"/>
+      <c r="AA1" s="35"/>
+      <c r="AB1" s="32"/>
+      <c r="AC1" s="32"/>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B2" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" s="18"/>
+      <c r="L2" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="M2" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="O2" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="P2" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q2" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="R2" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="S2" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U2" s="19"/>
+      <c r="V2" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="W2" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="X2" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y2" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="Z2" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="AA2" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="AB2" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC2" s="17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22"/>
+      <c r="U3" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="V3" s="21"/>
+      <c r="W3" s="21"/>
+      <c r="X3" s="22"/>
+      <c r="Y3" s="22"/>
+      <c r="Z3" s="22"/>
+      <c r="AA3" s="22"/>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B4" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="22">
+        <v>1818988686</v>
+      </c>
+      <c r="E4" s="22">
+        <v>1732622533</v>
+      </c>
+      <c r="F4" s="22">
+        <v>508605711</v>
+      </c>
+      <c r="G4" s="22">
+        <v>10</v>
+      </c>
+      <c r="H4" s="22">
+        <v>1327885248</v>
+      </c>
+      <c r="I4" s="22">
+        <v>3054046201</v>
+      </c>
+      <c r="K4" s="18"/>
+      <c r="L4" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M4" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="N4" s="22">
+        <v>1348609684</v>
+      </c>
+      <c r="O4" s="22">
+        <v>864830134</v>
+      </c>
+      <c r="P4" s="22">
+        <v>1167689544</v>
+      </c>
+      <c r="Q4" s="22">
+        <v>10</v>
+      </c>
+      <c r="R4" s="22">
+        <v>428234241</v>
+      </c>
+      <c r="S4" s="22">
+        <v>3704023741</v>
+      </c>
+      <c r="U4" s="24"/>
+      <c r="V4" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W4" s="21">
+        <v>1</v>
+      </c>
+      <c r="X4" s="22">
+        <v>2095632987.9000001</v>
+      </c>
+      <c r="Y4" s="22">
+        <v>811015351.39999998</v>
+      </c>
+      <c r="Z4" s="25">
+        <v>2446545000</v>
+      </c>
+      <c r="AA4" s="22">
+        <v>10</v>
+      </c>
+      <c r="AB4" s="25">
+        <v>325598700</v>
+      </c>
+      <c r="AC4" s="25">
+        <v>6535747000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B5" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="22">
+        <v>1507190719</v>
+      </c>
+      <c r="E5" s="22">
+        <v>1528807456</v>
+      </c>
+      <c r="F5" s="22">
+        <v>430334545</v>
+      </c>
+      <c r="G5" s="22">
+        <v>9</v>
+      </c>
+      <c r="H5" s="22">
+        <v>974082307</v>
+      </c>
+      <c r="I5" s="22">
+        <v>2344547966</v>
+      </c>
+      <c r="K5" s="18"/>
+      <c r="L5" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M5" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="N5" s="22">
+        <v>953918990</v>
+      </c>
+      <c r="O5" s="22">
+        <v>563925679</v>
+      </c>
+      <c r="P5" s="22">
+        <v>681710619</v>
+      </c>
+      <c r="Q5" s="22">
+        <v>9</v>
+      </c>
+      <c r="R5" s="22">
+        <v>429567818</v>
+      </c>
+      <c r="S5" s="22">
+        <v>2570666516</v>
+      </c>
+      <c r="U5" s="24"/>
+      <c r="V5" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W5" s="21">
+        <v>2</v>
+      </c>
+      <c r="X5" s="22">
+        <v>3947752322.8000002</v>
+      </c>
+      <c r="Y5" s="22">
+        <v>4008058228.9000001</v>
+      </c>
+      <c r="Z5" s="25">
+        <v>1802895000</v>
+      </c>
+      <c r="AA5" s="22">
+        <v>9</v>
+      </c>
+      <c r="AB5" s="25">
+        <v>1639683000</v>
+      </c>
+      <c r="AC5" s="25">
+        <v>6326754000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B6" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="22">
+        <v>1730519254</v>
+      </c>
+      <c r="E6" s="22">
+        <v>1457837646</v>
+      </c>
+      <c r="F6" s="22">
+        <v>1177081855</v>
+      </c>
+      <c r="G6" s="22">
+        <v>9</v>
+      </c>
+      <c r="H6" s="22">
+        <v>549846919</v>
+      </c>
+      <c r="I6" s="22">
+        <v>4466335682</v>
+      </c>
+      <c r="K6" s="18"/>
+      <c r="L6" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M6" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N6" s="22">
+        <v>1148559402</v>
+      </c>
+      <c r="O6" s="22">
+        <v>679562658</v>
+      </c>
+      <c r="P6" s="22">
+        <v>1071881602</v>
+      </c>
+      <c r="Q6" s="22">
+        <v>7</v>
+      </c>
+      <c r="R6" s="22">
+        <v>293307164</v>
+      </c>
+      <c r="S6" s="22">
+        <v>3279991055</v>
+      </c>
+      <c r="U6" s="24"/>
+      <c r="V6" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W6" s="21">
+        <v>3</v>
+      </c>
+      <c r="X6" s="22">
+        <v>4343170744.5</v>
+      </c>
+      <c r="Y6" s="22">
+        <v>4418865876.3999996</v>
+      </c>
+      <c r="Z6" s="25">
+        <v>2218956000</v>
+      </c>
+      <c r="AA6" s="22">
+        <v>9</v>
+      </c>
+      <c r="AB6" s="25">
+        <v>2371345000</v>
+      </c>
+      <c r="AC6" s="25">
+        <v>9466111000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B7" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="22">
+        <v>1726376444</v>
+      </c>
+      <c r="E7" s="22">
+        <v>1377994441</v>
+      </c>
+      <c r="F7" s="22">
+        <v>1441375972</v>
+      </c>
+      <c r="G7" s="22">
+        <v>9</v>
+      </c>
+      <c r="H7" s="22">
+        <v>478091032</v>
+      </c>
+      <c r="I7" s="22">
+        <v>5223338928</v>
+      </c>
+      <c r="K7" s="18"/>
+      <c r="L7" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M7" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="N7" s="22">
+        <v>5519552759</v>
+      </c>
+      <c r="O7" s="22">
+        <v>5519552759</v>
+      </c>
+      <c r="P7" s="22">
+        <v>7259004449</v>
+      </c>
+      <c r="Q7" s="22">
+        <v>2</v>
+      </c>
+      <c r="R7" s="22">
+        <v>386661489</v>
+      </c>
+      <c r="S7" s="22">
+        <v>10652444030</v>
+      </c>
+      <c r="U7" s="24"/>
+      <c r="V7" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W7" s="21">
+        <v>4</v>
+      </c>
+      <c r="X7" s="22">
+        <v>5743387443.6000004</v>
+      </c>
+      <c r="Y7" s="22">
+        <v>5152011880.1000004</v>
+      </c>
+      <c r="Z7" s="25">
+        <v>2797377000</v>
+      </c>
+      <c r="AA7" s="22">
+        <v>8</v>
+      </c>
+      <c r="AB7" s="25">
+        <v>1983194000</v>
+      </c>
+      <c r="AC7" s="25">
+        <v>11405760000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B8" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="22">
+        <v>1523821705</v>
+      </c>
+      <c r="E8" s="22">
+        <v>1440536379</v>
+      </c>
+      <c r="F8" s="22">
+        <v>610412973</v>
+      </c>
+      <c r="G8" s="22">
+        <v>9</v>
+      </c>
+      <c r="H8" s="22">
+        <v>897731555</v>
+      </c>
+      <c r="I8" s="22">
+        <v>2865709096</v>
+      </c>
+      <c r="K8" s="18"/>
+      <c r="L8" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M8" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="N8" s="22">
+        <v>1067030063</v>
+      </c>
+      <c r="O8" s="22">
+        <v>1014346146</v>
+      </c>
+      <c r="P8" s="22">
+        <v>640433269</v>
+      </c>
+      <c r="Q8" s="22">
+        <v>7</v>
+      </c>
+      <c r="R8" s="22">
+        <v>119972357</v>
+      </c>
+      <c r="S8" s="22">
+        <v>1832533895</v>
+      </c>
+      <c r="U8" s="24"/>
+      <c r="V8" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W8" s="21">
+        <v>1</v>
+      </c>
+      <c r="X8" s="22">
+        <v>244295.6</v>
+      </c>
+      <c r="Y8" s="22">
+        <v>198539.3</v>
+      </c>
+      <c r="Z8" s="25">
+        <v>192716.9</v>
+      </c>
+      <c r="AA8" s="22">
+        <v>6</v>
+      </c>
+      <c r="AB8" s="25">
+        <v>51414.47</v>
+      </c>
+      <c r="AC8" s="25">
+        <v>488056.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B9" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="22">
+        <v>1715452613</v>
+      </c>
+      <c r="E9" s="22">
+        <v>1015701000</v>
+      </c>
+      <c r="F9" s="22">
+        <v>1923798297</v>
+      </c>
+      <c r="G9" s="22">
+        <v>9</v>
+      </c>
+      <c r="H9" s="22">
+        <v>603735391</v>
+      </c>
+      <c r="I9" s="22">
+        <v>6765171727</v>
+      </c>
+      <c r="K9" s="18"/>
+      <c r="L9" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M9" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="N9" s="22">
+        <v>553990365</v>
+      </c>
+      <c r="O9" s="22">
+        <v>580496140</v>
+      </c>
+      <c r="P9" s="22">
+        <v>549184977</v>
+      </c>
+      <c r="Q9" s="22">
+        <v>7</v>
+      </c>
+      <c r="R9" s="22">
+        <v>-378614664</v>
+      </c>
+      <c r="S9" s="22">
+        <v>1354266114</v>
+      </c>
+      <c r="U9" s="24"/>
+      <c r="V9" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W9" s="21">
+        <v>2</v>
+      </c>
+      <c r="X9" s="22">
+        <v>210537.60000000001</v>
+      </c>
+      <c r="Y9" s="22">
+        <v>194384</v>
+      </c>
+      <c r="Z9" s="25">
+        <v>54685.02</v>
+      </c>
+      <c r="AA9" s="22">
+        <v>7</v>
+      </c>
+      <c r="AB9" s="25">
+        <v>142328.20000000001</v>
+      </c>
+      <c r="AC9" s="25">
+        <v>319663.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B10" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="22">
+        <v>2824148902</v>
+      </c>
+      <c r="E10" s="22">
+        <v>2263294113</v>
+      </c>
+      <c r="F10" s="22">
+        <v>1491108170</v>
+      </c>
+      <c r="G10" s="22">
+        <v>7</v>
+      </c>
+      <c r="H10" s="22">
+        <v>1282931409</v>
+      </c>
+      <c r="I10" s="22">
+        <v>5017210796</v>
+      </c>
+      <c r="K10" s="18"/>
+      <c r="L10" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M10" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N10" s="22">
+        <v>1256875143</v>
+      </c>
+      <c r="O10" s="22">
+        <v>989625712</v>
+      </c>
+      <c r="P10" s="22">
+        <v>932084386</v>
+      </c>
+      <c r="Q10" s="22">
+        <v>6</v>
+      </c>
+      <c r="R10" s="22">
+        <v>269801912</v>
+      </c>
+      <c r="S10" s="22">
+        <v>2683763834</v>
+      </c>
+      <c r="U10" s="24"/>
+      <c r="V10" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W10" s="21">
+        <v>3</v>
+      </c>
+      <c r="X10" s="22">
+        <v>249707.5</v>
+      </c>
+      <c r="Y10" s="22">
+        <v>244608.3</v>
+      </c>
+      <c r="Z10" s="25">
+        <v>72382.55</v>
+      </c>
+      <c r="AA10" s="22">
+        <v>6</v>
+      </c>
+      <c r="AB10" s="25">
+        <v>149720</v>
+      </c>
+      <c r="AC10" s="25">
+        <v>370641.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B11" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="22">
+        <v>2207934486</v>
+      </c>
+      <c r="E11" s="22">
+        <v>2207934486</v>
+      </c>
+      <c r="F11" s="22">
+        <v>938879269</v>
+      </c>
+      <c r="G11" s="22">
+        <v>2</v>
+      </c>
+      <c r="H11" s="22">
+        <v>1544046588</v>
+      </c>
+      <c r="I11" s="22">
+        <v>2871822383</v>
+      </c>
+      <c r="K11" s="18"/>
+      <c r="L11" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M11" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="N11" s="22">
+        <v>124165072</v>
+      </c>
+      <c r="O11" s="22">
+        <v>56727223</v>
+      </c>
+      <c r="P11" s="22">
+        <v>787225971</v>
+      </c>
+      <c r="Q11" s="22">
+        <v>6</v>
+      </c>
+      <c r="R11" s="22">
+        <v>-842862074</v>
+      </c>
+      <c r="S11" s="22">
+        <v>1312691981</v>
+      </c>
+      <c r="U11" s="24"/>
+      <c r="V11" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W11" s="21">
+        <v>4</v>
+      </c>
+      <c r="X11" s="22">
+        <v>300059.8</v>
+      </c>
+      <c r="Y11" s="22">
+        <v>257523.3</v>
+      </c>
+      <c r="Z11" s="25">
+        <v>80785.48</v>
+      </c>
+      <c r="AA11" s="22">
+        <v>7</v>
+      </c>
+      <c r="AB11" s="25">
+        <v>222664.7</v>
+      </c>
+      <c r="AC11" s="25">
+        <v>405537.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B12" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="22">
+        <v>524854242</v>
+      </c>
+      <c r="E12" s="22">
+        <v>299566058</v>
+      </c>
+      <c r="F12" s="22">
+        <v>452186958</v>
+      </c>
+      <c r="G12" s="22">
+        <v>7</v>
+      </c>
+      <c r="H12" s="22">
+        <v>216164385</v>
+      </c>
+      <c r="I12" s="22">
+        <v>1488517865</v>
+      </c>
+      <c r="K12" s="18"/>
+      <c r="U12" s="18"/>
+      <c r="V12" s="21"/>
+      <c r="W12" s="21"/>
+      <c r="X12" s="22"/>
+      <c r="Y12" s="22"/>
+      <c r="Z12" s="25"/>
+      <c r="AA12" s="22"/>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B13" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="22">
+        <v>451667037</v>
+      </c>
+      <c r="E13" s="22">
+        <v>516318922</v>
+      </c>
+      <c r="F13" s="22">
+        <v>253313505</v>
+      </c>
+      <c r="G13" s="22">
+        <v>7</v>
+      </c>
+      <c r="H13" s="22">
+        <v>149475253</v>
+      </c>
+      <c r="I13" s="22">
+        <v>883750566</v>
+      </c>
+      <c r="K13" s="18"/>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="K14" s="18"/>
+      <c r="L14" s="22"/>
+      <c r="M14" s="22"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="18"/>
+      <c r="P14" s="18"/>
+      <c r="Q14" s="18"/>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A15" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
+      <c r="U15" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="V15" s="21"/>
+      <c r="W15" s="21"/>
+      <c r="X15" s="22"/>
+      <c r="Y15" s="22"/>
+      <c r="Z15" s="25"/>
+      <c r="AA15" s="22"/>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B16" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C16" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="28">
+        <v>0.56888733400000002</v>
+      </c>
+      <c r="E16" s="28">
+        <v>0.60737149700000004</v>
+      </c>
+      <c r="F16" s="28">
+        <v>0.15037728</v>
+      </c>
+      <c r="G16" s="28">
+        <v>10</v>
+      </c>
+      <c r="H16" s="28">
+        <v>0.29098048199999998</v>
+      </c>
+      <c r="K16" s="18"/>
+      <c r="L16" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M16" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="N16" s="22">
+        <v>1.5337998580000001</v>
+      </c>
+      <c r="O16" s="22">
+        <v>1.1293449879999999</v>
+      </c>
+      <c r="P16" s="22">
+        <v>0.80901577000000002</v>
+      </c>
+      <c r="Q16" s="22">
+        <v>10</v>
+      </c>
+      <c r="R16" s="22">
+        <v>0.74831552499999998</v>
+      </c>
+      <c r="S16" s="22">
+        <v>3.1718225499999999</v>
+      </c>
+      <c r="U16" s="18"/>
+      <c r="V16" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W16" s="21">
+        <v>1</v>
+      </c>
+      <c r="X16" s="25">
+        <v>3.272433E-4</v>
+      </c>
+      <c r="Y16" s="25">
+        <v>1.156248E-4</v>
+      </c>
+      <c r="Z16" s="25">
+        <v>3.497226E-4</v>
+      </c>
+      <c r="AA16" s="22">
+        <v>10</v>
+      </c>
+      <c r="AB16" s="25">
+        <v>8.5070860000000003E-5</v>
+      </c>
+      <c r="AC16" s="25">
+        <v>9.7520289999999997E-4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B17" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="28">
+        <v>0.47287408199999997</v>
+      </c>
+      <c r="E17" s="28">
+        <v>0.53031773599999998</v>
+      </c>
+      <c r="F17" s="28">
+        <v>0.11331449</v>
+      </c>
+      <c r="G17" s="28">
+        <v>9</v>
+      </c>
+      <c r="H17" s="28">
+        <v>0.27573533</v>
+      </c>
+      <c r="K17" s="18"/>
+      <c r="L17" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M17" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="N17" s="22">
+        <v>1.2591298529999999</v>
+      </c>
+      <c r="O17" s="22">
+        <v>1.076509857</v>
+      </c>
+      <c r="P17" s="22">
+        <v>0.56466307000000004</v>
+      </c>
+      <c r="Q17" s="22">
+        <v>9</v>
+      </c>
+      <c r="R17" s="22">
+        <v>0.75064587599999999</v>
+      </c>
+      <c r="S17" s="22">
+        <v>2.2256950400000002</v>
+      </c>
+      <c r="U17" s="18"/>
+      <c r="V17" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W17" s="21">
+        <v>2</v>
+      </c>
+      <c r="X17" s="25">
+        <v>5.6137289999999996E-4</v>
+      </c>
+      <c r="Y17" s="25">
+        <v>5.3030799999999995E-4</v>
+      </c>
+      <c r="Z17" s="25">
+        <v>2.4492900000000001E-4</v>
+      </c>
+      <c r="AA17" s="22">
+        <v>9</v>
+      </c>
+      <c r="AB17" s="25">
+        <v>2.8365159999999999E-4</v>
+      </c>
+      <c r="AC17" s="25">
+        <v>1.0363099999999999E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B18" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C18" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="28">
+        <v>0.391756463</v>
+      </c>
+      <c r="E18" s="28">
+        <v>0.37492580399999997</v>
+      </c>
+      <c r="F18" s="28">
+        <v>8.5357810000000006E-2</v>
+      </c>
+      <c r="G18" s="28">
+        <v>9</v>
+      </c>
+      <c r="H18" s="28">
+        <v>0.28539893599999999</v>
+      </c>
+      <c r="K18" s="18"/>
+      <c r="L18" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M18" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N18" s="22">
+        <v>1.1331385540000001</v>
+      </c>
+      <c r="O18" s="22">
+        <v>0.89496726999999998</v>
+      </c>
+      <c r="P18" s="22">
+        <v>0.65686573999999998</v>
+      </c>
+      <c r="Q18" s="22">
+        <v>7</v>
+      </c>
+      <c r="R18" s="22">
+        <v>0.657925129</v>
+      </c>
+      <c r="S18" s="22">
+        <v>2.4464534800000002</v>
+      </c>
+      <c r="U18" s="18"/>
+      <c r="V18" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W18" s="21">
+        <v>3</v>
+      </c>
+      <c r="X18" s="25">
+        <v>2.795656E-4</v>
+      </c>
+      <c r="Y18" s="25">
+        <v>2.5580900000000002E-4</v>
+      </c>
+      <c r="Z18" s="25">
+        <v>6.9616049999999996E-5</v>
+      </c>
+      <c r="AA18" s="22">
+        <v>9</v>
+      </c>
+      <c r="AB18" s="25">
+        <v>2.0475429999999999E-4</v>
+      </c>
+      <c r="AC18" s="25">
+        <v>4.0080619999999998E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B19" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C19" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="28">
+        <v>0.36728765699999999</v>
+      </c>
+      <c r="E19" s="28">
+        <v>0.32373421200000002</v>
+      </c>
+      <c r="F19" s="28">
+        <v>0.10424920999999999</v>
+      </c>
+      <c r="G19" s="28">
+        <v>9</v>
+      </c>
+      <c r="H19" s="28">
+        <v>0.28164594199999998</v>
+      </c>
+      <c r="K19" s="18"/>
+      <c r="L19" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M19" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="N19" s="22">
+        <v>1.2922687770000001</v>
+      </c>
+      <c r="O19" s="22">
+        <v>1.2922687770000001</v>
+      </c>
+      <c r="P19" s="22">
+        <v>1.27514862</v>
+      </c>
+      <c r="Q19" s="22">
+        <v>2</v>
+      </c>
+      <c r="R19" s="22">
+        <v>0.39060254100000003</v>
+      </c>
+      <c r="S19" s="22">
+        <v>2.1939350100000001</v>
+      </c>
+      <c r="U19" s="18"/>
+      <c r="V19" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W19" s="21">
+        <v>4</v>
+      </c>
+      <c r="X19" s="25">
+        <v>1.6145459999999999E-4</v>
+      </c>
+      <c r="Y19" s="25">
+        <v>1.6796960000000001E-4</v>
+      </c>
+      <c r="Z19" s="25">
+        <v>5.742336E-5</v>
+      </c>
+      <c r="AA19" s="22">
+        <v>8</v>
+      </c>
+      <c r="AB19" s="25">
+        <v>8.2952139999999998E-5</v>
+      </c>
+      <c r="AC19" s="25">
+        <v>2.5859480000000001E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B20" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C20" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="28">
+        <v>0.242342961</v>
+      </c>
+      <c r="E20" s="28">
+        <v>0.22425549</v>
+      </c>
+      <c r="F20" s="28">
+        <v>6.2626340000000003E-2</v>
+      </c>
+      <c r="G20" s="28">
+        <v>9</v>
+      </c>
+      <c r="H20" s="28">
+        <v>0.16837772100000001</v>
+      </c>
+      <c r="K20" s="18"/>
+      <c r="L20" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M20" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="N20" s="22">
+        <v>6.5850077000000007E-2</v>
+      </c>
+      <c r="O20" s="22">
+        <v>2.9983362E-2</v>
+      </c>
+      <c r="P20" s="22">
+        <v>7.4472789999999997E-2</v>
+      </c>
+      <c r="Q20" s="22">
+        <v>7</v>
+      </c>
+      <c r="R20" s="22">
+        <v>7.6323119999999996E-3</v>
+      </c>
+      <c r="S20" s="22">
+        <v>0.21598027</v>
+      </c>
+      <c r="U20" s="18"/>
+      <c r="V20" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W20" s="21">
+        <v>1</v>
+      </c>
+      <c r="X20" s="25">
+        <v>1.8620549999999999E-5</v>
+      </c>
+      <c r="Y20" s="25">
+        <v>1.1060870000000001E-5</v>
+      </c>
+      <c r="Z20" s="25">
+        <v>2.1393690000000001E-5</v>
+      </c>
+      <c r="AA20" s="22">
+        <v>6</v>
+      </c>
+      <c r="AB20" s="25">
+        <v>6.5416939999999998E-6</v>
+      </c>
+      <c r="AC20" s="25">
+        <v>6.2097620000000001E-5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B21" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="28">
+        <v>0.19818725200000001</v>
+      </c>
+      <c r="E21" s="28">
+        <v>0.17759317199999999</v>
+      </c>
+      <c r="F21" s="28">
+        <v>6.2059919999999998E-2</v>
+      </c>
+      <c r="G21" s="28">
+        <v>9</v>
+      </c>
+      <c r="H21" s="28">
+        <v>0.12320901200000001</v>
+      </c>
+      <c r="K21" s="18"/>
+      <c r="L21" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M21" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="N21" s="22">
+        <v>3.4482240999999997E-2</v>
+      </c>
+      <c r="O21" s="22">
+        <v>3.6929569000000002E-2</v>
+      </c>
+      <c r="P21" s="22">
+        <v>3.3258959999999997E-2</v>
+      </c>
+      <c r="Q21" s="22">
+        <v>7</v>
+      </c>
+      <c r="R21" s="22">
+        <v>-1.1615752E-2</v>
+      </c>
+      <c r="S21" s="22">
+        <v>8.6154690000000006E-2</v>
+      </c>
+      <c r="U21" s="18"/>
+      <c r="V21" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W21" s="21">
+        <v>2</v>
+      </c>
+      <c r="X21" s="25">
+        <v>2.0778410000000002E-5</v>
+      </c>
+      <c r="Y21" s="25">
+        <v>1.961431E-5</v>
+      </c>
+      <c r="Z21" s="25">
+        <v>5.4055409999999998E-6</v>
+      </c>
+      <c r="AA21" s="22">
+        <v>7</v>
+      </c>
+      <c r="AB21" s="25">
+        <v>1.289266E-5</v>
+      </c>
+      <c r="AC21" s="25">
+        <v>2.8903449999999999E-5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B22" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C22" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="28">
+        <v>0.23649199000000001</v>
+      </c>
+      <c r="E22" s="28">
+        <v>0.27307756</v>
+      </c>
+      <c r="F22" s="28">
+        <v>6.9391610000000006E-2</v>
+      </c>
+      <c r="G22" s="28">
+        <v>7</v>
+      </c>
+      <c r="H22" s="28">
+        <v>0.108911085</v>
+      </c>
+      <c r="K22" s="18"/>
+      <c r="L22" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M22" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N22" s="22">
+        <v>4.0041553000000001E-2</v>
+      </c>
+      <c r="O22" s="22">
+        <v>3.0361336999999999E-2</v>
+      </c>
+      <c r="P22" s="22">
+        <v>2.689325E-2</v>
+      </c>
+      <c r="Q22" s="22">
+        <v>6</v>
+      </c>
+      <c r="R22" s="22">
+        <v>1.6486554E-2</v>
+      </c>
+      <c r="S22" s="22">
+        <v>8.2336839999999994E-2</v>
+      </c>
+      <c r="U22" s="18"/>
+      <c r="V22" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W22" s="21">
+        <v>3</v>
+      </c>
+      <c r="X22" s="25">
+        <v>1.696567E-5</v>
+      </c>
+      <c r="Y22" s="25">
+        <v>1.5886060000000001E-5</v>
+      </c>
+      <c r="Z22" s="25">
+        <v>3.4255029999999999E-6</v>
+      </c>
+      <c r="AA22" s="22">
+        <v>6</v>
+      </c>
+      <c r="AB22" s="25">
+        <v>1.333608E-5</v>
+      </c>
+      <c r="AC22" s="25">
+        <v>2.274229E-5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B23" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="28">
+        <v>0.169330227</v>
+      </c>
+      <c r="E23" s="28">
+        <v>0.169330227</v>
+      </c>
+      <c r="F23" s="28">
+        <v>6.2682059999999998E-2</v>
+      </c>
+      <c r="G23" s="28">
+        <v>2</v>
+      </c>
+      <c r="H23" s="28">
+        <v>0.12500732000000001</v>
+      </c>
+      <c r="K23" s="18"/>
+      <c r="L23" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M23" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="N23" s="22">
+        <v>7.9013580000000007E-3</v>
+      </c>
+      <c r="O23" s="22">
+        <v>1.649675E-3</v>
+      </c>
+      <c r="P23" s="22">
+        <v>1.9280820000000001E-2</v>
+      </c>
+      <c r="Q23" s="22">
+        <v>6</v>
+      </c>
+      <c r="R23" s="22">
+        <v>-1.0591717E-2</v>
+      </c>
+      <c r="S23" s="22">
+        <v>4.0272889999999999E-2</v>
+      </c>
+      <c r="U23" s="18"/>
+      <c r="V23" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W23" s="21">
+        <v>4</v>
+      </c>
+      <c r="X23" s="25">
+        <v>1.5223910000000001E-5</v>
+      </c>
+      <c r="Y23" s="25">
+        <v>1.4090439999999999E-5</v>
+      </c>
+      <c r="Z23" s="25">
+        <v>4.68868E-6</v>
+      </c>
+      <c r="AA23" s="22">
+        <v>7</v>
+      </c>
+      <c r="AB23" s="25">
+        <v>1.0069380000000001E-5</v>
+      </c>
+      <c r="AC23" s="25">
+        <v>2.1744100000000001E-5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B24" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="28">
+        <v>3.7079503E-2</v>
+      </c>
+      <c r="E24" s="28">
+        <v>1.5590998999999999E-2</v>
+      </c>
+      <c r="F24" s="28">
+        <v>6.1286130000000001E-2</v>
+      </c>
+      <c r="G24" s="28">
+        <v>7</v>
+      </c>
+      <c r="H24" s="28">
+        <v>6.0299339999999998E-3</v>
+      </c>
+      <c r="U24" s="18"/>
+      <c r="V24" s="18"/>
+      <c r="W24" s="18"/>
+      <c r="X24" s="18"/>
+      <c r="Y24" s="18"/>
+      <c r="Z24" s="18"/>
+      <c r="AA24" s="18"/>
+    </row>
+    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B25" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="22">
+        <v>2.1694549E-2</v>
+      </c>
+      <c r="E25" s="22">
+        <v>1.6327897000000001E-2</v>
+      </c>
+      <c r="F25" s="22">
+        <v>1.086296E-2</v>
+      </c>
+      <c r="G25" s="22">
+        <v>7</v>
+      </c>
+      <c r="H25" s="22">
+        <v>6.7141329999999997E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="K26" s="18"/>
+      <c r="L26" s="22"/>
+      <c r="M26" s="22"/>
+      <c r="N26" s="22"/>
+      <c r="O26" s="18"/>
+      <c r="P26" s="18"/>
+      <c r="Q26" s="18"/>
+    </row>
+    <row r="27" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A27" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="H27" s="29"/>
+      <c r="K27" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="L27" s="18"/>
+      <c r="M27" s="18"/>
+      <c r="N27" s="18"/>
+      <c r="O27" s="18"/>
+      <c r="P27" s="18"/>
+      <c r="Q27" s="18"/>
+      <c r="U27" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="V27" s="18"/>
+      <c r="W27" s="18"/>
+      <c r="X27" s="18"/>
+      <c r="Y27" s="18"/>
+      <c r="Z27" s="18"/>
+      <c r="AA27" s="18"/>
+    </row>
+    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B28" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="28">
+        <v>1.42221833</v>
+      </c>
+      <c r="E28" s="28">
+        <v>1.5184287400000001</v>
+      </c>
+      <c r="F28" s="28">
+        <v>0.37594319999999998</v>
+      </c>
+      <c r="G28" s="28">
+        <v>10</v>
+      </c>
+      <c r="H28" s="28">
+        <v>0.72745121000000001</v>
+      </c>
+      <c r="K28" s="18"/>
+      <c r="L28" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M28" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="N28" s="22">
+        <v>1.9172498</v>
+      </c>
+      <c r="O28" s="22">
+        <v>1.4116812350000001</v>
+      </c>
+      <c r="P28" s="22">
+        <v>1.0112697100000001</v>
+      </c>
+      <c r="Q28" s="22">
+        <v>10</v>
+      </c>
+      <c r="R28" s="22">
+        <v>0.93539441000000001</v>
+      </c>
+      <c r="S28" s="22">
+        <v>3.9647782</v>
+      </c>
+      <c r="U28" s="18"/>
+      <c r="V28" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W28" s="21">
+        <v>1</v>
+      </c>
+      <c r="X28" s="22">
+        <v>5.5982293999999998E-3</v>
+      </c>
+      <c r="Y28" s="22">
+        <v>1.8463842E-3</v>
+      </c>
+      <c r="Z28" s="25">
+        <v>6.2629649999999997E-3</v>
+      </c>
+      <c r="AA28" s="22">
+        <v>10</v>
+      </c>
+      <c r="AB28" s="22">
+        <v>1.4939216E-3</v>
+      </c>
+      <c r="AC28" s="22">
+        <v>1.6482528199999999E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B29" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C29" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="28">
+        <v>1.1821852100000001</v>
+      </c>
+      <c r="E29" s="28">
+        <v>1.3257943400000001</v>
+      </c>
+      <c r="F29" s="28">
+        <v>0.28328621999999998</v>
+      </c>
+      <c r="G29" s="28">
+        <v>9</v>
+      </c>
+      <c r="H29" s="28">
+        <v>0.68933833</v>
+      </c>
+      <c r="K29" s="18"/>
+      <c r="L29" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M29" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="N29" s="22">
+        <v>1.5739122999999999</v>
+      </c>
+      <c r="O29" s="22">
+        <v>1.3456373210000001</v>
+      </c>
+      <c r="P29" s="22">
+        <v>0.70582884000000001</v>
+      </c>
+      <c r="Q29" s="22">
+        <v>9</v>
+      </c>
+      <c r="R29" s="22">
+        <v>0.93830734999999998</v>
+      </c>
+      <c r="S29" s="22">
+        <v>2.7821188000000001</v>
+      </c>
+      <c r="U29" s="18"/>
+      <c r="V29" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W29" s="21">
+        <v>2</v>
+      </c>
+      <c r="X29" s="22">
+        <v>1.13823495E-2</v>
+      </c>
+      <c r="Y29" s="22">
+        <v>1.00058118E-2</v>
+      </c>
+      <c r="Z29" s="25">
+        <v>5.2308889999999999E-3</v>
+      </c>
+      <c r="AA29" s="22">
+        <v>9</v>
+      </c>
+      <c r="AB29" s="22">
+        <v>5.3821774999999999E-3</v>
+      </c>
+      <c r="AC29" s="22">
+        <v>2.2528481400000001E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B30" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="28">
+        <v>0.97939116000000004</v>
+      </c>
+      <c r="E30" s="28">
+        <v>0.93731450999999999</v>
+      </c>
+      <c r="F30" s="28">
+        <v>0.21339451000000001</v>
+      </c>
+      <c r="G30" s="28">
+        <v>9</v>
+      </c>
+      <c r="H30" s="28">
+        <v>0.71349733999999998</v>
+      </c>
+      <c r="K30" s="18"/>
+      <c r="L30" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M30" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N30" s="22">
+        <v>1.4164232000000001</v>
+      </c>
+      <c r="O30" s="22">
+        <v>1.118709087</v>
+      </c>
+      <c r="P30" s="22">
+        <v>0.82108217999999999</v>
+      </c>
+      <c r="Q30" s="22">
+        <v>7</v>
+      </c>
+      <c r="R30" s="22">
+        <v>0.82240641000000003</v>
+      </c>
+      <c r="S30" s="22">
+        <v>3.0580668000000002</v>
+      </c>
+      <c r="U30" s="18"/>
+      <c r="V30" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W30" s="21">
+        <v>3</v>
+      </c>
+      <c r="X30" s="22">
+        <v>5.4730513000000001E-3</v>
+      </c>
+      <c r="Y30" s="22">
+        <v>5.0158618999999998E-3</v>
+      </c>
+      <c r="Z30" s="25">
+        <v>1.379269E-3</v>
+      </c>
+      <c r="AA30" s="22">
+        <v>9</v>
+      </c>
+      <c r="AB30" s="22">
+        <v>4.0950850999999996E-3</v>
+      </c>
+      <c r="AC30" s="22">
+        <v>8.0161230999999996E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B31" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="28">
+        <v>0.91821914000000004</v>
+      </c>
+      <c r="E31" s="28">
+        <v>0.80933553000000003</v>
+      </c>
+      <c r="F31" s="28">
+        <v>0.26062302999999998</v>
+      </c>
+      <c r="G31" s="28">
+        <v>9</v>
+      </c>
+      <c r="H31" s="28">
+        <v>0.70411484999999996</v>
+      </c>
+      <c r="K31" s="18"/>
+      <c r="L31" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M31" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="N31" s="22">
+        <v>1.6153360000000001</v>
+      </c>
+      <c r="O31" s="22">
+        <v>1.6153359709999999</v>
+      </c>
+      <c r="P31" s="22">
+        <v>1.5939357700000001</v>
+      </c>
+      <c r="Q31" s="22">
+        <v>2</v>
+      </c>
+      <c r="R31" s="22">
+        <v>0.48825318000000001</v>
+      </c>
+      <c r="S31" s="22">
+        <v>2.7424187999999998</v>
+      </c>
+      <c r="U31" s="18"/>
+      <c r="V31" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W31" s="21">
+        <v>4</v>
+      </c>
+      <c r="X31" s="22">
+        <v>3.0512158999999998E-3</v>
+      </c>
+      <c r="Y31" s="22">
+        <v>3.2277482E-3</v>
+      </c>
+      <c r="Z31" s="25">
+        <v>1.0148900000000001E-3</v>
+      </c>
+      <c r="AA31" s="22">
+        <v>8</v>
+      </c>
+      <c r="AB31" s="22">
+        <v>1.6021360000000001E-3</v>
+      </c>
+      <c r="AC31" s="22">
+        <v>4.7887918999999996E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B32" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C32" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="28">
+        <v>0.60585739999999999</v>
+      </c>
+      <c r="E32" s="28">
+        <v>0.56063872999999997</v>
+      </c>
+      <c r="F32" s="28">
+        <v>0.15656586</v>
+      </c>
+      <c r="G32" s="28">
+        <v>9</v>
+      </c>
+      <c r="H32" s="28">
+        <v>0.42094429999999999</v>
+      </c>
+      <c r="K32" s="18"/>
+      <c r="L32" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M32" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="N32" s="22">
+        <v>0.1646252</v>
+      </c>
+      <c r="O32" s="22">
+        <v>7.4958406000000005E-2</v>
+      </c>
+      <c r="P32" s="22">
+        <v>0.18618198</v>
+      </c>
+      <c r="Q32" s="22">
+        <v>7</v>
+      </c>
+      <c r="R32" s="22">
+        <v>1.9080779999999999E-2</v>
+      </c>
+      <c r="S32" s="22">
+        <v>0.53995070000000001</v>
+      </c>
+      <c r="U32" s="18"/>
+      <c r="V32" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W32" s="21">
+        <v>1</v>
+      </c>
+      <c r="X32" s="22">
+        <v>7.9428479999999997E-4</v>
+      </c>
+      <c r="Y32" s="22">
+        <v>4.0558670000000001E-4</v>
+      </c>
+      <c r="Z32" s="25">
+        <v>9.9621249999999996E-4</v>
+      </c>
+      <c r="AA32" s="22">
+        <v>6</v>
+      </c>
+      <c r="AB32" s="22">
+        <v>2.6166779999999999E-4</v>
+      </c>
+      <c r="AC32" s="22">
+        <v>2.8226191999999998E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B33" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C33" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="28">
+        <v>0.49546813000000001</v>
+      </c>
+      <c r="E33" s="28">
+        <v>0.44398293</v>
+      </c>
+      <c r="F33" s="28">
+        <v>0.1551498</v>
+      </c>
+      <c r="G33" s="28">
+        <v>9</v>
+      </c>
+      <c r="H33" s="28">
+        <v>0.30802253000000002</v>
+      </c>
+      <c r="K33" s="18"/>
+      <c r="L33" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M33" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="N33" s="22">
+        <v>8.6205599999999993E-2</v>
+      </c>
+      <c r="O33" s="22">
+        <v>9.2323922000000003E-2</v>
+      </c>
+      <c r="P33" s="22">
+        <v>8.3147399999999996E-2</v>
+      </c>
+      <c r="Q33" s="22">
+        <v>7</v>
+      </c>
+      <c r="R33" s="22">
+        <v>-2.903938E-2</v>
+      </c>
+      <c r="S33" s="22">
+        <v>0.21538669999999999</v>
+      </c>
+      <c r="U33" s="18"/>
+      <c r="V33" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W33" s="21">
+        <v>2</v>
+      </c>
+      <c r="X33" s="22">
+        <v>4.35213E-4</v>
+      </c>
+      <c r="Y33" s="22">
+        <v>4.065284E-4</v>
+      </c>
+      <c r="Z33" s="25">
+        <v>1.6422029999999999E-4</v>
+      </c>
+      <c r="AA33" s="22">
+        <v>7</v>
+      </c>
+      <c r="AB33" s="22">
+        <v>2.8650360000000001E-4</v>
+      </c>
+      <c r="AC33" s="22">
+        <v>7.8117430000000003E-4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B34" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="28">
+        <v>0.59122998000000004</v>
+      </c>
+      <c r="E34" s="28">
+        <v>0.68269389999999996</v>
+      </c>
+      <c r="F34" s="28">
+        <v>0.17347902000000001</v>
+      </c>
+      <c r="G34" s="28">
+        <v>7</v>
+      </c>
+      <c r="H34" s="28">
+        <v>0.27227771000000001</v>
+      </c>
+      <c r="K34" s="18"/>
+      <c r="L34" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M34" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N34" s="22">
+        <v>0.1001039</v>
+      </c>
+      <c r="O34" s="22">
+        <v>7.5903340999999999E-2</v>
+      </c>
+      <c r="P34" s="22">
+        <v>6.7233130000000002E-2</v>
+      </c>
+      <c r="Q34" s="22">
+        <v>6</v>
+      </c>
+      <c r="R34" s="22">
+        <v>4.1216389999999999E-2</v>
+      </c>
+      <c r="S34" s="22">
+        <v>0.2058421</v>
+      </c>
+      <c r="U34" s="18"/>
+      <c r="V34" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W34" s="21">
+        <v>3</v>
+      </c>
+      <c r="X34" s="22">
+        <v>3.830897E-4</v>
+      </c>
+      <c r="Y34" s="22">
+        <v>3.8034309999999998E-4</v>
+      </c>
+      <c r="Z34" s="25">
+        <v>8.1128539999999997E-5</v>
+      </c>
+      <c r="AA34" s="22">
+        <v>6</v>
+      </c>
+      <c r="AB34" s="22">
+        <v>2.6672160000000002E-4</v>
+      </c>
+      <c r="AC34" s="22">
+        <v>5.1687010000000004E-4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B35" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="C35" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D35" s="28">
+        <v>0.42332556999999998</v>
+      </c>
+      <c r="E35" s="28">
+        <v>0.42332556999999998</v>
+      </c>
+      <c r="F35" s="28">
+        <v>0.15670513999999999</v>
+      </c>
+      <c r="G35" s="28">
+        <v>2</v>
+      </c>
+      <c r="H35" s="28">
+        <v>0.31251830000000003</v>
+      </c>
+      <c r="K35" s="18"/>
+      <c r="L35" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M35" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="N35" s="22">
+        <v>1.9753400000000001E-2</v>
+      </c>
+      <c r="O35" s="22">
+        <v>4.124188E-3</v>
+      </c>
+      <c r="P35" s="22">
+        <v>4.8202040000000002E-2</v>
+      </c>
+      <c r="Q35" s="22">
+        <v>6</v>
+      </c>
+      <c r="R35" s="22">
+        <v>-2.6479289999999999E-2</v>
+      </c>
+      <c r="S35" s="22">
+        <v>0.1006822</v>
+      </c>
+      <c r="U35" s="18"/>
+      <c r="V35" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W35" s="21">
+        <v>4</v>
+      </c>
+      <c r="X35" s="22">
+        <v>3.7532119999999998E-4</v>
+      </c>
+      <c r="Y35" s="22">
+        <v>3.8902259999999998E-4</v>
+      </c>
+      <c r="Z35" s="25">
+        <v>6.8401749999999996E-5</v>
+      </c>
+      <c r="AA35" s="22">
+        <v>7</v>
+      </c>
+      <c r="AB35" s="22">
+        <v>2.7325070000000002E-4</v>
+      </c>
+      <c r="AC35" s="22">
+        <v>4.5146949999999998E-4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B36" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="C36" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="28">
+        <v>0.18539752000000001</v>
+      </c>
+      <c r="E36" s="28">
+        <v>7.7954990000000002E-2</v>
+      </c>
+      <c r="F36" s="28">
+        <v>0.30643066000000002</v>
+      </c>
+      <c r="G36" s="28">
+        <v>7</v>
+      </c>
+      <c r="H36" s="28">
+        <v>3.014967E-2</v>
+      </c>
+      <c r="U36" s="18"/>
+      <c r="V36" s="18"/>
+      <c r="W36" s="18"/>
+      <c r="X36" s="18"/>
+      <c r="Y36" s="18"/>
+      <c r="Z36" s="18"/>
+      <c r="AA36" s="18"/>
+    </row>
+    <row r="37" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B37" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="22">
+        <v>0.10847274</v>
+      </c>
+      <c r="E37" s="22">
+        <v>8.163948E-2</v>
+      </c>
+      <c r="F37" s="22">
+        <v>5.431478E-2</v>
+      </c>
+      <c r="G37" s="22">
+        <v>7</v>
+      </c>
+      <c r="H37" s="22">
+        <v>3.3570669999999997E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A39" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="K39" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="L39" s="18"/>
+      <c r="M39" s="18"/>
+      <c r="N39" s="18"/>
+      <c r="O39" s="18"/>
+      <c r="P39" s="18"/>
+      <c r="Q39" s="18"/>
+      <c r="U39" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="V39" s="18"/>
+      <c r="W39" s="18"/>
+      <c r="X39" s="18"/>
+      <c r="Y39" s="18"/>
+      <c r="Z39" s="18"/>
+      <c r="AA39" s="18"/>
+    </row>
+    <row r="40" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B40" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="22">
+        <v>3.0321460600000001</v>
+      </c>
+      <c r="E40" s="22">
+        <v>3.0810997420000001</v>
+      </c>
+      <c r="F40" s="22">
+        <v>0.75162790000000002</v>
+      </c>
+      <c r="G40" s="22">
+        <v>10</v>
+      </c>
+      <c r="H40" s="22">
+        <v>1.8076861</v>
+      </c>
+      <c r="I40" s="24"/>
+      <c r="K40" s="22"/>
+      <c r="L40" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M40" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="N40" s="22">
+        <v>4.1983958250000004</v>
+      </c>
+      <c r="O40" s="22">
+        <v>3.2606717399999998</v>
+      </c>
+      <c r="P40" s="22">
+        <v>2.2010991</v>
+      </c>
+      <c r="Q40" s="22">
+        <v>10</v>
+      </c>
+      <c r="R40" s="22">
+        <v>1.81442025</v>
+      </c>
+      <c r="S40" s="22">
+        <v>8.7224999570000001</v>
+      </c>
+      <c r="U40" s="18"/>
+      <c r="V40" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W40" s="21">
+        <v>1</v>
+      </c>
+      <c r="X40" s="22">
+        <v>2.9313020000000002E-3</v>
+      </c>
+      <c r="Y40" s="22">
+        <v>9.6679600000000002E-4</v>
+      </c>
+      <c r="Z40" s="25">
+        <v>3.2793549999999999E-3</v>
+      </c>
+      <c r="AA40" s="22">
+        <v>10</v>
+      </c>
+      <c r="AB40" s="22">
+        <v>7.8224200000000005E-4</v>
+      </c>
+      <c r="AC40" s="22">
+        <v>8.6304390000000002E-3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B41" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C41" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="22">
+        <v>2.4038784099999999</v>
+      </c>
+      <c r="E41" s="22">
+        <v>2.6772074300000002</v>
+      </c>
+      <c r="F41" s="22">
+        <v>0.71126069999999997</v>
+      </c>
+      <c r="G41" s="22">
+        <v>9</v>
+      </c>
+      <c r="H41" s="22">
+        <v>1.2125984999999999</v>
+      </c>
+      <c r="I41" s="24"/>
+      <c r="K41" s="22"/>
+      <c r="L41" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M41" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="N41" s="22">
+        <v>3.043112523</v>
+      </c>
+      <c r="O41" s="22">
+        <v>2.9755895799999998</v>
+      </c>
+      <c r="P41" s="22">
+        <v>1.3639927000000001</v>
+      </c>
+      <c r="Q41" s="22">
+        <v>9</v>
+      </c>
+      <c r="R41" s="22">
+        <v>1.52184633</v>
+      </c>
+      <c r="S41" s="22">
+        <v>5.2447837699999997</v>
+      </c>
+      <c r="U41" s="18"/>
+      <c r="V41" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W41" s="21">
+        <v>2</v>
+      </c>
+      <c r="X41" s="22">
+        <v>5.9600186000000003E-3</v>
+      </c>
+      <c r="Y41" s="22">
+        <v>5.2391970000000001E-3</v>
+      </c>
+      <c r="Z41" s="25">
+        <v>2.7390029999999998E-3</v>
+      </c>
+      <c r="AA41" s="22">
+        <v>9</v>
+      </c>
+      <c r="AB41" s="22">
+        <v>2.818156E-3</v>
+      </c>
+      <c r="AC41" s="22">
+        <v>1.1796315E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B42" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42" s="22">
+        <v>2.0145505500000001</v>
+      </c>
+      <c r="E42" s="22">
+        <v>1.974890461</v>
+      </c>
+      <c r="F42" s="22">
+        <v>0.41716809999999999</v>
+      </c>
+      <c r="G42" s="22">
+        <v>9</v>
+      </c>
+      <c r="H42" s="22">
+        <v>1.3166682999999999</v>
+      </c>
+      <c r="I42" s="24"/>
+      <c r="K42" s="22"/>
+      <c r="L42" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M42" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N42" s="22">
+        <v>2.8960393450000002</v>
+      </c>
+      <c r="O42" s="22">
+        <v>2.3962959000000001</v>
+      </c>
+      <c r="P42" s="22">
+        <v>1.5578646</v>
+      </c>
+      <c r="Q42" s="22">
+        <v>7</v>
+      </c>
+      <c r="R42" s="22">
+        <v>1.70199506</v>
+      </c>
+      <c r="S42" s="22">
+        <v>6.1447794309999999</v>
+      </c>
+      <c r="U42" s="18"/>
+      <c r="V42" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W42" s="21">
+        <v>3</v>
+      </c>
+      <c r="X42" s="22">
+        <v>2.8657859999999999E-3</v>
+      </c>
+      <c r="Y42" s="22">
+        <v>2.6264019999999999E-3</v>
+      </c>
+      <c r="Z42" s="25">
+        <v>7.2221280000000002E-4</v>
+      </c>
+      <c r="AA42" s="22">
+        <v>9</v>
+      </c>
+      <c r="AB42" s="22">
+        <v>2.1442259999999999E-3</v>
+      </c>
+      <c r="AC42" s="22">
+        <v>4.1974029999999997E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B43" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C43" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" s="22">
+        <v>1.77225883</v>
+      </c>
+      <c r="E43" s="22">
+        <v>1.7542925110000001</v>
+      </c>
+      <c r="F43" s="22">
+        <v>0.48708940000000001</v>
+      </c>
+      <c r="G43" s="22">
+        <v>9</v>
+      </c>
+      <c r="H43" s="22">
+        <v>1.219897</v>
+      </c>
+      <c r="I43" s="24"/>
+      <c r="K43" s="22"/>
+      <c r="L43" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="M43" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="N43" s="22">
+        <v>2.7488906150000001</v>
+      </c>
+      <c r="O43" s="22">
+        <v>2.7488906100000001</v>
+      </c>
+      <c r="P43" s="22">
+        <v>3.2790845000000002</v>
+      </c>
+      <c r="Q43" s="22">
+        <v>2</v>
+      </c>
+      <c r="R43" s="22">
+        <v>0.43022770999999999</v>
+      </c>
+      <c r="S43" s="22">
+        <v>5.0675535170000003</v>
+      </c>
+      <c r="U43" s="18"/>
+      <c r="V43" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="W43" s="21">
+        <v>4</v>
+      </c>
+      <c r="X43" s="22">
+        <v>1.5976759999999999E-3</v>
+      </c>
+      <c r="Y43" s="22">
+        <v>1.6901144999999999E-3</v>
+      </c>
+      <c r="Z43" s="25">
+        <v>5.3142330000000005E-4</v>
+      </c>
+      <c r="AA43" s="22">
+        <v>8</v>
+      </c>
+      <c r="AB43" s="22">
+        <v>8.3889900000000005E-4</v>
+      </c>
+      <c r="AC43" s="22">
+        <v>2.5075140000000002E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B44" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" s="22">
+        <v>1.0856765900000001</v>
+      </c>
+      <c r="E44" s="22">
+        <v>1.063085676</v>
+      </c>
+      <c r="F44" s="22">
+        <v>0.28910720000000001</v>
+      </c>
+      <c r="G44" s="22">
+        <v>9</v>
+      </c>
+      <c r="H44" s="22">
+        <v>0.70033460000000003</v>
+      </c>
+      <c r="I44" s="24"/>
+      <c r="K44" s="22"/>
+      <c r="L44" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M44" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="N44" s="22">
+        <v>0.16416520600000001</v>
+      </c>
+      <c r="O44" s="22">
+        <v>-0.1140403</v>
+      </c>
+      <c r="P44" s="22">
+        <v>0.42127559999999997</v>
+      </c>
+      <c r="Q44" s="22">
+        <v>7</v>
+      </c>
+      <c r="R44" s="22">
+        <v>-0.19733654</v>
+      </c>
+      <c r="S44" s="22">
+        <v>0.79116838599999995</v>
+      </c>
+      <c r="U44" s="18"/>
+      <c r="V44" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W44" s="21">
+        <v>1</v>
+      </c>
+      <c r="X44" s="22">
+        <v>4.158993E-4</v>
+      </c>
+      <c r="Y44" s="22">
+        <v>2.1236949999999999E-4</v>
+      </c>
+      <c r="Z44" s="25">
+        <v>5.2164170000000001E-4</v>
+      </c>
+      <c r="AA44" s="22">
+        <v>6</v>
+      </c>
+      <c r="AB44" s="22">
+        <v>1.37009E-4</v>
+      </c>
+      <c r="AC44" s="22">
+        <v>1.4779859999999999E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B45" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C45" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="D45" s="22">
+        <v>0.89682479000000004</v>
+      </c>
+      <c r="E45" s="22">
+        <v>0.89394154999999997</v>
+      </c>
+      <c r="F45" s="22">
+        <v>0.29041529999999999</v>
+      </c>
+      <c r="G45" s="22">
+        <v>9</v>
+      </c>
+      <c r="H45" s="22">
+        <v>0.55313049999999997</v>
+      </c>
+      <c r="I45" s="24"/>
+      <c r="K45" s="22"/>
+      <c r="L45" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M45" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="N45" s="22">
+        <v>3.8959580000000001E-3</v>
+      </c>
+      <c r="O45" s="22">
+        <v>3.1547609999999997E-2</v>
+      </c>
+      <c r="P45" s="22">
+        <v>0.2174923</v>
+      </c>
+      <c r="Q45" s="22">
+        <v>7</v>
+      </c>
+      <c r="R45" s="22">
+        <v>-0.26293989000000001</v>
+      </c>
+      <c r="S45" s="22">
+        <v>0.30396409699999999</v>
+      </c>
+      <c r="U45" s="18"/>
+      <c r="V45" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W45" s="21">
+        <v>2</v>
+      </c>
+      <c r="X45" s="22">
+        <v>2.1631609999999999E-4</v>
+      </c>
+      <c r="Y45" s="22">
+        <v>2.1052399999999999E-4</v>
+      </c>
+      <c r="Z45" s="25">
+        <v>6.1282879999999994E-5</v>
+      </c>
+      <c r="AA45" s="22">
+        <v>7</v>
+      </c>
+      <c r="AB45" s="22">
+        <v>1.50013E-4</v>
+      </c>
+      <c r="AC45" s="22">
+        <v>3.3608200000000003E-4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B46" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C46" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="D46" s="22">
+        <v>1.1477364699999999</v>
+      </c>
+      <c r="E46" s="22">
+        <v>1.2726616740000001</v>
+      </c>
+      <c r="F46" s="22">
+        <v>0.31281720000000002</v>
+      </c>
+      <c r="G46" s="22">
+        <v>7</v>
+      </c>
+      <c r="H46" s="22">
+        <v>0.54615910000000001</v>
+      </c>
+      <c r="I46" s="24"/>
+      <c r="K46" s="22"/>
+      <c r="L46" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M46" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N46" s="22">
+        <v>3.9487002E-2</v>
+      </c>
+      <c r="O46" s="22">
+        <v>2.040525E-2</v>
+      </c>
+      <c r="P46" s="22">
+        <v>0.1189621</v>
+      </c>
+      <c r="Q46" s="22">
+        <v>6</v>
+      </c>
+      <c r="R46" s="22">
+        <v>-7.2314829999999997E-2</v>
+      </c>
+      <c r="S46" s="22">
+        <v>0.248740655</v>
+      </c>
+      <c r="U46" s="18"/>
+      <c r="V46" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W46" s="21">
+        <v>3</v>
+      </c>
+      <c r="X46" s="22">
+        <v>2.0058629999999999E-4</v>
+      </c>
+      <c r="Y46" s="22">
+        <v>1.991475E-4</v>
+      </c>
+      <c r="Z46" s="25">
+        <v>4.2479209999999999E-5</v>
+      </c>
+      <c r="AA46" s="22">
+        <v>6</v>
+      </c>
+      <c r="AB46" s="22">
+        <v>1.3965700000000001E-4</v>
+      </c>
+      <c r="AC46" s="22">
+        <v>2.7063500000000003E-4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B47" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="22">
+        <v>0.80843693000000005</v>
+      </c>
+      <c r="E47" s="22">
+        <v>0.80843692700000003</v>
+      </c>
+      <c r="F47" s="22">
+        <v>0.31152790000000002</v>
+      </c>
+      <c r="G47" s="22">
+        <v>2</v>
+      </c>
+      <c r="H47" s="22">
+        <v>0.58815340000000005</v>
+      </c>
+      <c r="I47" s="24"/>
+      <c r="K47" s="22"/>
+      <c r="L47" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="M47" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="N47" s="22">
+        <v>-0.21236607900000001</v>
+      </c>
+      <c r="O47" s="22">
+        <v>-0.21916107000000001</v>
+      </c>
+      <c r="P47" s="22">
+        <v>0.1298716</v>
+      </c>
+      <c r="Q47" s="22">
+        <v>6</v>
+      </c>
+      <c r="R47" s="22">
+        <v>-0.39258610999999999</v>
+      </c>
+      <c r="S47" s="22">
+        <v>-1.042666E-3</v>
+      </c>
+      <c r="U47" s="18"/>
+      <c r="V47" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="W47" s="21">
+        <v>4</v>
+      </c>
+      <c r="X47" s="22">
+        <v>1.9578489999999999E-4</v>
+      </c>
+      <c r="Y47" s="22">
+        <v>2.0369100000000001E-4</v>
+      </c>
+      <c r="Z47" s="25">
+        <v>3.6849920000000002E-5</v>
+      </c>
+      <c r="AA47" s="22">
+        <v>7</v>
+      </c>
+      <c r="AB47" s="22">
+        <v>1.4307400000000001E-4</v>
+      </c>
+      <c r="AC47" s="22">
+        <v>2.3639700000000001E-4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="B48" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D48" s="22">
+        <v>0.22171249000000001</v>
+      </c>
+      <c r="E48" s="22">
+        <v>-4.9050829999999997E-2</v>
+      </c>
+      <c r="F48" s="22">
+        <v>0.70884069999999999</v>
+      </c>
+      <c r="G48" s="22">
+        <v>7</v>
+      </c>
+      <c r="H48" s="22">
+        <v>-0.13965240000000001</v>
+      </c>
+      <c r="I48" s="24"/>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B49" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49" s="22">
+        <v>5.7967369999999997E-2</v>
+      </c>
+      <c r="E49" s="22">
+        <v>1.19051E-4</v>
+      </c>
+      <c r="F49" s="22">
+        <v>0.19997239999999999</v>
+      </c>
+      <c r="G49" s="22">
+        <v>7</v>
+      </c>
+      <c r="H49" s="22">
+        <v>-0.22707830000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>